<commit_message>
Add temporary files for Shamil Nabiyev's review
</commit_message>
<xml_diff>
--- a/mylift_onreview_government.xlsx
+++ b/mylift_onreview_government.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -658,22 +658,22 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>683</t>
+          <t>666</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>SA-KT-MR</t>
+          <t>TKJ1000/1.5</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>SHANGHAI  SURAPID  INTERNATIONAL TRADE CO.,LTD</t>
+          <t>Huzhou Fuji Elevator Co., LTD</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>RL25081501YL- L3</t>
+          <t>AZE18009</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -683,17 +683,17 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>AZ. KOMFORT MMC - bina №37a</t>
+          <t>"Gold Qayalı" Market</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Seymur Orucov Küçəsi, 47, Bakı, Azərbaycan</t>
+          <t>İsmət Qayıbov Küçəsi, Sumqayıt, Azərbaycan</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2025-09-12</t>
+          <t>2018-04-27</t>
         </is>
       </c>
       <c r="I4" s="2" t="n">
@@ -701,34 +701,34 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>https://storage.mylift.az/mylift/lift_683_a5a24_passport.pdf?v=66408e32</t>
+          <t>https://storage.mylift.az/mylift/lift_666_8a617_passport.pdf?v=678fe4bf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>682</t>
+          <t>663</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>SA-KT-MR</t>
+          <t>TKJ1000/1.5</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>SHANGHAI  SURAPID  INTERNATIONAL TRADE CO.,LTD</t>
+          <t>Huzhou Fuji Elevator Co., LTD</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>RL25081501YL- L2</t>
+          <t>AZE18008</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -738,17 +738,17 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>AZ. KOMFORT MMC - bina №37a</t>
+          <t>"Gold Qayalı" Market</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Seymur Orucov Küçəsi, 47, Bakı, Azərbaycan</t>
+          <t>İsmət Qayıbov Küçəsi, Sumqayıt, Azərbaycan</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>2025-09-12</t>
+          <t>2018-04-27</t>
         </is>
       </c>
       <c r="I5" s="3" t="n">
@@ -756,34 +756,34 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>https://storage.mylift.az/mylift/lift_682_a53a9_passport.pdf?v=500204bf</t>
+          <t>https://storage.mylift.az/mylift/lift_663_85eaf_passport.pdf?v=760b6a29</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>681</t>
+          <t>628</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>SA-KT-MR</t>
+          <t>BLT-QS(CHOI-III)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>SHANGHAI  SURAPID  INTERNATIONAL TRADE CO.,LTD</t>
+          <t>BLT BRILLIANT,Shenyang Yuanda Intellectual Industry Group CO.,LTD (BLT ELEVATOR)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>RL25081501YL- L4</t>
+          <t>BLTSY23K/00865</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -793,17 +793,17 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>AZ. KOMFORT MMC - bina №37a</t>
+          <t>ŞİNKAR HOLDİNG</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Seymur Orucov Küçəsi, 47, Bakı, Azərbaycan</t>
+          <t>Bakı, Azərbaycan</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>2025-09-12</t>
+          <t>2023-05-28</t>
         </is>
       </c>
       <c r="I6" s="2" t="n">
@@ -811,34 +811,34 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>https://storage.mylift.az/mylift/lift_681_a352a_passport.pdf?v=439eec24</t>
+          <t>https://storage.mylift.az/mylift/lift_628_9b0ac_passport.pdf?v=1aadfaf6</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>679</t>
+          <t>622</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>SA-KT-MR</t>
+          <t>AP (450/1.0-JXW)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>SHANGHAI  SURAPID  INTERNATIONAL TRADE CO.,LTD</t>
+          <t>AUX EXPRESS (SUZHOU) ELEVATOR CO.,LTD</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>RL25081501YL- L1</t>
+          <t>A2507053</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -848,17 +848,17 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>AZ. KOMFORT MMC - bina №37a</t>
+          <t>Neman IKF</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Seymur Orucov Küçəsi, 47, Bakı, Azərbaycan</t>
+          <t>Baksol Küçəsi, Bakı, Azərbaycan</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>2025-09-12</t>
+          <t>2025-08-29</t>
         </is>
       </c>
       <c r="I7" s="3" t="n">
@@ -866,34 +866,34 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>https://storage.mylift.az/mylift/lift_679_a11b0_passport.pdf?v=be983229</t>
+          <t>https://storage.mylift.az/mylift/lift_622_6c900_passport.pdf?v=1d5d1f06</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>628</t>
+          <t>511</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>BLT-QS(CHOI-III)</t>
+          <t>OTİS</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>BLT BRILLIANT,Shenyang Yuanda Intellectual Industry Group CO.,LTD (BLT ELEVATOR)</t>
+          <t>XIZI OTİS ELEVATOR CO.,LTD</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>BLTSY23K/00865</t>
+          <t>B7NZ5436</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -903,17 +903,17 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>ŞİNKAR HOLDİNG</t>
+          <t>"Chukur Qabala Museum Hotel" MMC</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Bakı, Azərbaycan</t>
+          <t>Çuxur Qəbələ, Qəbələ, Azərbaycan</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2023-05-28</t>
+          <t>2014-12-31</t>
         </is>
       </c>
       <c r="I8" s="2" t="n">
@@ -921,54 +921,50 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>https://storage.mylift.az/mylift/lift_628_9b0ac_passport.pdf?v=1aadfaf6</t>
-        </is>
-      </c>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>622</t>
+          <t>421</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>AP (450/1.0-JXW)</t>
+          <t>MR</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>AUX EXPRESS (SUZHOU) ELEVATOR CO.,LTD</t>
+          <t>Moris Elevator Co.,Ltd</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>A2507053</t>
+          <t>177568</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>electric</t>
+          <t>hydraulic</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Neman IKF</t>
+          <t>Vego Hotel</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Baksol Küçəsi, Bakı, Azərbaycan</t>
+          <t>Gəncə, Azərbaycan</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>2025-08-29</t>
+          <t>2013-05-14</t>
         </is>
       </c>
       <c r="I9" s="3" t="n">
@@ -976,54 +972,50 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="K9" s="3" t="inlineStr">
-        <is>
-          <t>https://storage.mylift.az/mylift/lift_622_6c900_passport.pdf?v=1d5d1f06</t>
-        </is>
-      </c>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>511</t>
+          <t>420</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>OTİS</t>
+          <t>MR</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>XIZI OTİS ELEVATOR CO.,LTD</t>
+          <t>Moris Elevator Co.,Ltd</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>B7NZ5436</t>
+          <t>177567</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>electric</t>
+          <t>hydraulic</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>"Chukur Qabala Museum Hotel" MMC</t>
+          <t>Vego Hotel</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Çuxur Qəbələ, Qəbələ, Azərbaycan</t>
+          <t>Gəncə, Azərbaycan</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>2014-12-31</t>
+          <t>2013-05-14</t>
         </is>
       </c>
       <c r="I10" s="2" t="n">
@@ -1031,7 +1023,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr"/>
@@ -1039,22 +1031,22 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>432</t>
+          <t>412</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>GeN2</t>
+          <t xml:space="preserve">N MonoSpace				</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>OTIS ELEVATOR CO.,LTD</t>
+          <t>KONE Elevators Co Ltd,</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>2018Q1NAN908</t>
+          <t xml:space="preserve">45388604 		 		</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1064,17 +1056,17 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>"SEBA FİTO TİBB" MMC</t>
+          <t>Akhundov Office</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Neftçilər Prospekti, Bakı, Azərbaycan</t>
+          <t>Nizami Gəncəvi Küçəsi, 149, Bakı, Azərbaycan</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>2018-03-08</t>
+          <t>2024-01-03</t>
         </is>
       </c>
       <c r="I11" s="3" t="n">
@@ -1082,19 +1074,19 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>https://storage.mylift.az/mylift/lift_432_8ddb6_passport.pdf?v=3881b38f</t>
+          <t>https://storage.mylift.az/mylift/lift_412_87bde_passport.pdf?v=e42ee87f</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>421</t>
+          <t>351</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1109,7 +1101,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>177568</t>
+          <t>177577</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1137,7 +1129,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -1145,42 +1137,42 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>420</t>
+          <t>083</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>MR</t>
+          <t>NZR</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Moris Elevator Co.,Ltd</t>
+          <t>Nazar Döküm Hidrolik Galvaniz Asansör ve Kuyumculuk Sanayi ve Ticaret Limited Şirketi</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>177567</t>
+          <t>NZR-2022-230</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>hydraulic</t>
+          <t>electric</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Vego Hotel</t>
+          <t>"Boulevard Medical Center"</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Gəncə, Azərbaycan</t>
+          <t>Sumqayıt, Azərbaycan</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>2013-05-14</t>
+          <t>2022-05-09</t>
         </is>
       </c>
       <c r="I13" s="3" t="n">
@@ -1188,30 +1180,34 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="inlineStr"/>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>https://storage.mylift.az/mylift/lift_083_bfc60_passport.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>412</t>
+          <t>061</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N MonoSpace				</t>
+          <t>Enta villa</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>KONE Elevators Co Ltd,</t>
+          <t>TK Elevator China Co. Ltd</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">45388604 		 		</t>
+          <t>L0MO 029138.001</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1221,72 +1217,72 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Akhundov Office</t>
+          <t>Qazax ADA Tələbə Evi</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Nizami Gəncəvi Küçəsi, 149, Bakı, Azərbaycan</t>
+          <t>Qazax, Azərbaycan</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2024-01-03</t>
+          <t>2024-05-31</t>
         </is>
       </c>
       <c r="I14" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>https://storage.mylift.az/mylift/lift_412_87bde_passport.pdf?v=e42ee87f</t>
+          <t>https://storage.mylift.az/mylift/lift_061_87286_passport.pdf?v=4e667a8b</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>351</t>
+          <t>047</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>MR</t>
+          <t>SİGMA</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Moris Elevator Co.,Ltd</t>
+          <t>Korea Respublikası</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>177577</t>
+          <t>2010BE 0163E01-1</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>hydraulic</t>
+          <t>electric</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Vego Hotel</t>
+          <t>"Der Mond" Hotel</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Gəncə, Azərbaycan</t>
+          <t>Sütəmurdov, Lənkəran, Azərbaycan</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>2013-05-14</t>
+          <t>2010-02-22</t>
         </is>
       </c>
       <c r="I15" s="3" t="n">
@@ -1294,30 +1290,34 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
-        </is>
-      </c>
-      <c r="K15" s="3" t="inlineStr"/>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>https://storage.mylift.az/mylift/lift_047_8ff7b_passport.pdf?v=ebfdc2ee</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>083</t>
+          <t>017</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>NZR</t>
+          <t>TKJW800</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Nazar Döküm Hidrolik Galvaniz Asansör ve Kuyumculuk Sanayi ve Ticaret Limited Şirketi</t>
+          <t>Fuji</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>NZR-2022-230</t>
+          <t>JL-XS-TRS-20241015-10</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1327,17 +1327,17 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>"Boulevard Medical Center"</t>
+          <t xml:space="preserve">Monte Napoleone Hotel </t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Sumqayıt, Azərbaycan</t>
+          <t>Nəsib bəy Yusifbəyli Prospekti, 84, Bakı, Azərbaycan</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>2022-05-09</t>
+          <t>2024-02-10</t>
         </is>
       </c>
       <c r="I16" s="2" t="n">
@@ -1345,34 +1345,30 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>https://storage.mylift.az/mylift/lift_083_bfc60_passport.pdf</t>
-        </is>
-      </c>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>078</t>
+          <t>016</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>MR</t>
+          <t>TKJW800</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>TOSHIBA ELEVATOR CO., LTD</t>
+          <t>Fuji</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>2020-ST-03</t>
+          <t>24010585</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1382,52 +1378,48 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Sea Tower</t>
+          <t xml:space="preserve">Monte Napoleone Hotel </t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>2-cı Fəvarələr Küçəsi, Baku, Azerbaijan</t>
+          <t>Nəsib bəy Yusifbəyli Prospekti, 84, Bakı, Azərbaycan</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>2020-04-15</t>
+          <t>2024-02-10</t>
         </is>
       </c>
       <c r="I17" s="3" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
-        </is>
-      </c>
-      <c r="K17" s="3" t="inlineStr">
-        <is>
-          <t>https://storage.mylift.az/mylift/lift_078_b2943_passport.pdf?v=2d5e7c20</t>
-        </is>
-      </c>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>077</t>
+          <t>015</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>MR</t>
+          <t>TKJW800</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>TOSHIBA ELEVATOR CO., LTD</t>
+          <t>Fuji</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2020-ST-02</t>
+          <t>24042869</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1437,17 +1429,17 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Sea Tower</t>
+          <t xml:space="preserve">Monte Napoleone Hotel </t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>2-cı Fəvarələr Küçəsi, Baku, Azerbaijan</t>
+          <t>Nəsib bəy Yusifbəyli Prospekti, 84, Bakı, Azərbaycan</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2020-04-15</t>
+          <t>2024-02-10</t>
         </is>
       </c>
       <c r="I18" s="2" t="n">
@@ -1455,332 +1447,10 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>https://storage.mylift.az/mylift/lift_077_b2902_passport.pdf?v=7ca041a9</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>076</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>MR</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>TOSHIBA ELEVATOR CO., LTD</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>2020-ST-01</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>electric</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Sea Tower</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>2-cı Fəvarələr Küçəsi, Baku, Azerbaijan</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>2020-04-15</t>
-        </is>
-      </c>
-      <c r="I19" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="J19" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-14</t>
-        </is>
-      </c>
-      <c r="K19" s="3" t="inlineStr">
-        <is>
-          <t>https://storage.mylift.az/mylift/lift_076_b1a19_passport.pdf?v=694e1216</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>061</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Enta villa</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>TK Elevator China Co. Ltd</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>L0MO 029138.001</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>electric</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Qazax ADA Tələbə Evi</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>Qazax, Azərbaycan</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>2024-05-31</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-13</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>https://storage.mylift.az/mylift/lift_061_87286_passport.pdf?v=4e667a8b</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>047</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>SİGMA</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Korea Respublikası</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>2010BE 0163E01-1</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>electric</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>"Der Mond" Hotel</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>Sütəmurdov, Lənkəran, Azərbaycan</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>2010-02-22</t>
-        </is>
-      </c>
-      <c r="I21" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-09</t>
-        </is>
-      </c>
-      <c r="K21" s="3" t="inlineStr">
-        <is>
-          <t>https://storage.mylift.az/mylift/lift_047_8ff7b_passport.pdf?v=ebfdc2ee</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>017</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>TKJW800</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Fuji</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>JL-XS-TRS-20241015-10</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>electric</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Monte Napoleone Hotel </t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>Nəsib bəy Yusifbəyli Prospekti, 84, Bakı, Azərbaycan</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>2024-02-10</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-19</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>016</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>TKJW800</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>Fuji</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>24010585</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>electric</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Monte Napoleone Hotel </t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>Nəsib bəy Yusifbəyli Prospekti, 84, Bakı, Azərbaycan</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>2024-02-10</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="J23" s="3" t="inlineStr">
-        <is>
           <t>2026-02-10</t>
         </is>
       </c>
-      <c r="K23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>015</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>TKJW800</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Fuji</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>24042869</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>electric</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Monte Napoleone Hotel </t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>Nəsib bəy Yusifbəyli Prospekti, 84, Bakı, Azərbaycan</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>2024-02-10</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-10</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1819,7 +1489,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -1842,7 +1512,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>19.06.2026 14:19</t>
+          <t>23.06.2026 09:58</t>
         </is>
       </c>
     </row>

</xml_diff>